<commit_message>
The UAT workbook explains each module's workflow, not only its steps
Testers could follow a case's steps without knowing why the module exists,
what it needs first or what it leaves for the next one, which makes a bug
and a deliberate behaviour hard to tell apart.

uat-guide.mjs holds one entry per module: what it proves, its screens, who
signs in, the workflow in five or six steps, what it needs first, what it
leaves ready, the setup it needs and a time estimate. Three places read it:
a new Module Guide sheet, a one-line summary on every module band in Test
Cases, and a diagram on the Read Me sheet drawn by build-diagram.mjs with
the Chromium Playwright already installed for the e2e suite.

The whole run is about 710 minutes, summed by formula on the guide sheet.
UAT_OUT lets the builder write elsewhere while Excel holds the file open.

Signed-off-by: agungksidik <agungksidik@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/testing/OpenOKR-UAT.xlsx
+++ b/docs/testing/OpenOKR-UAT.xlsx
@@ -6,14 +6,15 @@
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="1" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" r:id="rId2"/>
-    <sheet name="Personas" sheetId="3" r:id="rId3"/>
-    <sheet name="Test Cases" sheetId="4" r:id="rId4"/>
-    <sheet name="Bug Log" sheetId="5" r:id="rId5"/>
+    <sheet name="Module Guide" sheetId="2" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" r:id="rId3"/>
+    <sheet name="Personas" sheetId="4" r:id="rId4"/>
+    <sheet name="Test Cases" sheetId="5" r:id="rId5"/>
+    <sheet name="Bug Log" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Test Cases'!$A$1:$N$216</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Bug Log'!$A$1:$M$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test Cases'!$A$1:$N$216</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Bug Log'!$A$1:$M$62</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -108,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -131,6 +132,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -193,6 +197,44 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="8382000" cy="7439025"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Workflow" descr="The order to test the modules in, from set up to integrations"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="8382000" cy="7439025"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
@@ -223,357 +265,1947 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">The workflow at a glance</t>
+        </is>
+      </c>
+      <c r="B4" s="2"/>
+    </row>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52">
+      <c r="A52" s="9"/>
+      <c r="B52" s="9"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">How to use this workbook</t>
         </is>
       </c>
-      <c r="B4" s="2"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="1">
+      <c r="B53" s="2"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="1">
         <v>1</v>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B54" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Start a fresh instance with an empty database (docs/install/compose.md). Note the URL.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1">
+    <row r="55">
+      <c r="A55" s="1">
         <v>2</v>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B55" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Fill the yellow email and password cells on the Personas sheet.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1">
+    <row r="56">
+      <c r="A56" s="1">
         <v>3</v>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B56" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Work down the Test Cases sheet in order. Each module builds on the one before it.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1">
+    <row r="57">
+      <c r="A57" s="1">
         <v>4</v>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B57" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Sign in as the person in "Login as". Check the Pre-condition, follow the Steps, compare with Expected result.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1">
+    <row r="58">
+      <c r="A58" s="1">
         <v>5</v>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B58" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Pick a Status from the dropdown. For anything other than Pass, write what you saw in "Actual result / notes".</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1">
+    <row r="59">
+      <c r="A59" s="1">
         <v>6</v>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B59" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">For each Fail or Error, add a row on Bug Log with a screenshot link, and put its Bug ID on the test case.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1">
+    <row r="60">
+      <c r="A60" s="1">
         <v>7</v>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B60" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Read the Summary sheet for the totals. It updates by itself.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="9"/>
+      <c r="B61" s="9"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Status</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">When to use it</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not Run</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="B63" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Not tested yet. Every case starts here.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B64" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">What you saw matches Expected result.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B65" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">The screen works but the result is different from Expected result. Wrong text, wrong number, missing item, a refusal that should not happen.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Error</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B66" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">The app broke: an error page, "We could not load", a blank screen, a spinner that never ends, or a crash.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Blocked</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B67" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">You could not run the test because something earlier failed, or a pre-condition cannot be met. Say which in the notes.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="B19" s="1" t="inlineStr">
+      <c r="B68" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Does not apply to this instance, for example no Slack workspace or no passkey device.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="9"/>
+      <c r="B69" s="9"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Before you start</t>
         </is>
       </c>
-      <c r="B21" s="2"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="B70" s="2"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Browsers</t>
         </is>
       </c>
-      <c r="B22" s="1" t="inlineStr">
+      <c r="B71" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">One browser profile per persona. Two screens help for M13 and M15, where two people act at once.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Email</t>
         </is>
       </c>
-      <c r="B23" s="1" t="inlineStr">
+      <c r="B72" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Without SMTP the instance prints every mail to its log. Invitation links are also shown once on Admin, Invitations. For reset links either read the server log or run Mailpit (SMTP on localhost port 1025, inbox at http://localhost:8025).</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Server access</t>
         </is>
       </c>
-      <c r="B24" s="1" t="inlineStr">
+      <c r="B73" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">A few cases need someone who can read logs, restart the instance or run a pnpm command. They say so in the hint.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">AI</t>
         </is>
       </c>
-      <c r="B25" s="1" t="inlineStr">
+      <c r="B74" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">AI is off by default and everything before M20 is tested with it off. M20 needs a provider key with a spending limit.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Integrations</t>
         </is>
       </c>
-      <c r="B26" s="1" t="inlineStr">
+      <c r="B75" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">M21 to M26 need outside accounts (Slack, Teams, WhatsApp, Telegram, an identity provider, an MCP client). Mark N/A for any you do not have.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Never</t>
         </is>
       </c>
-      <c r="B27" s="1" t="inlineStr">
+      <c r="B76" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Paste an API key, token or password into this workbook. Write where it is kept instead.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="9"/>
-      <c r="B28" s="9"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="9"/>
+      <c r="B77" s="9"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Known risks found while writing this</t>
         </is>
       </c>
-      <c r="B29" s="2"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+      <c r="B78" s="2"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Publishing</t>
         </is>
       </c>
-      <c r="B30" s="1" t="inlineStr">
+      <c r="B79" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Code review suggests gates 2 and 5 have no field in the UI. M11-05 tests it. If they cannot turn green, publish with the override in M11-07.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Sessions</t>
         </is>
       </c>
-      <c r="B31" s="1" t="inlineStr">
+      <c r="B80" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Sessions cannot be created from the UI. The only weekly session is the one the starter template makes in M02. Quarterly reviews may not be reachable at all (M18-06).</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Admins</t>
         </is>
       </c>
-      <c r="B32" s="1" t="inlineStr">
+      <c r="B81" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Only the first account has full access, and no screen grants it to anyone else.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Chat test</t>
         </is>
       </c>
-      <c r="B33" s="1" t="inlineStr">
+      <c r="B82" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">"Send me a test" on Admin, Channels sends an email, not a chat message.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">2FA</t>
         </is>
       </c>
-      <c r="B34" s="1" t="inlineStr">
+      <c r="B83" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">There is no button to turn one-time codes off. Use the throwaway persona Amara.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="9"/>
-      <c r="B35" s="9"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Generated from docs/testing/uat-cases.mjs. 189 test cases across 26 modules.</t>
-        </is>
-      </c>
-      <c r="B36" s="10"/>
+    <row r="84">
+      <c r="A84" s="9"/>
+      <c r="B84" s="9"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generated from docs/testing/uat-cases.mjs and uat-guide.mjs. 189 test cases across 26 modules.</t>
+        </is>
+      </c>
+      <c r="B85" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="13">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="A69:B69"/>
+    <mergeCell ref="A70:B70"/>
+    <mergeCell ref="A77:B77"/>
+    <mergeCell ref="A78:B78"/>
+    <mergeCell ref="A84:B84"/>
+    <mergeCell ref="A85:B85"/>
+  </mergeCells>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="30" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="50" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="34" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="10" max="10" width="9" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What each module is for and how it flows, in the order to test it. The Test Cases sheet has the detailed steps; this sheet is the map.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phase</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What it proves</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Screens</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Who signs in</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workflow</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Needs first</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leaves ready for later</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Setup needed</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Time (min)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M01 Install and first account</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Set up</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turn an empty server into an instance with one owner</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/setup, /setup/account, /sign-up</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open the instance and get sent to setup
+2. Name the instance Northwind Labs
+3. Create the owner account
+4. Check that registration is now closed</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nothing. Start here</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An owner account. Everybody after this joins by invitation</t>
+        </is>
+      </c>
+      <c r="I5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A fresh instance with an empty database</t>
+        </is>
+      </c>
+      <c r="J5" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" ht="71" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M02 Welcome wizard</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Set up</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Give the new workspace its name, clock, rhythm and starting content</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/welcome</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Name the workspace and pick its timezone
+2. Choose the check-in rhythm
+3. Skip the invite
+4. Apply the OKR starter cycle template
+5. Land on the work map</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M01</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A current cycle, one objective with 3 key results, a KPI, a KPI tree and the weekly session M15 needs</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nothing extra</t>
+        </is>
+      </c>
+      <c r="J6" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" ht="71" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M03 Workspace settings</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Set up</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check that workspace settings save, reload and reset</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin: General, Branding, Rhythm and thresholds</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Change timezone and language
+2. Check the mail warning
+3. Set a brand colour
+4. Set the check-in rhythm
+5. Rename a concept, then set it back</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M02</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The rhythm every later reminder and due date follows</t>
+        </is>
+      </c>
+      <c r="I7" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nothing extra</t>
+        </is>
+      </c>
+      <c r="J7" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" ht="97" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M04 Invitations and building the team</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2. Build the team</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bring the seven Northwind people into the workspace</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin, Invitations; /join/&lt;token&gt;; /sign-up</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin, then each persona</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Admin creates a personal invitation for Priya
+2. Priya opens the link and signs up
+3. A wrong address is refused
+4. Admin shares one link for the rest
+5. Each persona signs up in their own browser profile
+6. Revoked and made-up links are refused</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M02</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eight members. Every module after this signs in as one of them</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One inbox with plus-addresses, one browser profile per persona</t>
+        </is>
+      </c>
+      <c r="J8" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" ht="84" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M05 Sign-in and account security</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2. Build the team</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prove sign-in, password reset and the second factor protect an account</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/sign-in, /forgot-password, /reset-password, /backup-code, Account, Security</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jonas, Mei, Amara, Sara, Priya</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Refuse a wrong password
+2. Reset a forgotten password by mail
+3. Turn on one-time codes for Amara
+4. Sign in with a code and with a backup code
+5. Add a passkey
+6. Revoke another device</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M04</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confidence that accounts are safe before real data goes in</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mailpit or SMTP for the reset mail. An authenticator app</t>
+        </is>
+      </c>
+      <c r="J9" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" ht="71" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M06 People and org chart</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2. Build the team</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Give everyone a title and a manager so the org chart is real</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">People, People / &lt;person&gt;</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin, Mei, Jonas, Tomas</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Admin sets title and manager for each persona
+2. Check the org chart
+3. A loop in the chain is refused
+4. Members edit only their own profile
+5. Suspend and restore Tomas</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M04</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reporting lines, used by the org chart and by who reviews whom</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nothing extra</t>
+        </is>
+      </c>
+      <c r="J10" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" ht="71" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M07 Spaces</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2. Build the team</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Create the team homes that own goals, boards and sessions</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spaces, Spaces / &lt;space&gt;</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin, Priya, Amara, Jonas</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Admin creates Product, Sales and Customer Success
+2. Priya adds members with roles
+3. A member joins and leaves
+4. A non-manager cannot manage
+5. Change settings, archive a spare space</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M06</t>
+        </is>
+      </c>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spaces that goals, the board and the weekly session belong to</t>
+        </is>
+      </c>
+      <c r="I11" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nothing extra</t>
+        </is>
+      </c>
+      <c r="J11" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" ht="84" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M08 Cycle: prepare, diagnose, direction</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Plan the cycle</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Walk the first three phases so drafting has something to stand on</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle (phases 1 to 3), Cycles card</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin, Priya</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Read the eight-phase rail
+2. Create the next cycle and set the publication deadline
+3. Phase 1: sponsor, facilitator, input pack
+4. Phase 2: rank three strategic issues
+5. Phase 3: choose a priority</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M07</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A priority for objectives to contribute to, and the deadline gate 6 checks</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nothing extra</t>
+        </is>
+      </c>
+      <c r="J12" s="1">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" ht="84" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M09 Drafting OKRs and quality checks</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Plan the cycle</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Draft objectives and key results while the quality checks fire live</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle, phase 4; /method/&lt;rule&gt;</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sara, Daniel, Tomas</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Draft Sara's objective with champion and reviewer
+2. Type weak wording and watch OBJ-1 and OBJ-2 fire
+3. Open a rule card and the method page
+4. Add key results, weak then measurable
+5. Record a current value
+6. Daniel and Tomas draft their own</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M08</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A draft set of objectives for three teams</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AI off</t>
+        </is>
+      </c>
+      <c r="J13" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" ht="97" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M10 Goal page and documents</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Plan the cycle</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Work on one goal: values, confidence, comments, documents and files</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Goals, Goals / &lt;goal&gt;, Documents / &lt;doc&gt;</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sara, Priya, Mei, Jonas</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open the goal and read its header
+2. Update values and confidence
+3. Comment and watch
+4. Start a private document, then publish two versions
+5. Attach and detach a file
+6. Filter the explorer</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M09</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A goal with history, discussion and a document</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A small PDF to attach</t>
+        </is>
+      </c>
+      <c r="J14" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" ht="84" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M11 Alignment and publishing</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Plan the cycle</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Align the set and publish it through the six gates</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Goals, Alignment studio; Cycle, phase 5</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Priya, Admin</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Look at the cascade
+2. Link a team goal to the company goal
+3. Record and confirm a dependency
+4. Read each gate and follow its fix
+5. Publish, or override with a reason
+6. Check a member cannot publish</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M10</t>
+        </is>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A published set. The cycle moves to phase 6 and check-ins start</t>
+        </is>
+      </c>
+      <c r="I15" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nothing extra</t>
+        </is>
+      </c>
+      <c r="J15" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" ht="84" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M12 KPIs and recovery</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Run the cycle</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Track KPIs continuously and recover one that falls out of its corridor</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KPIs grid, KPIs / &lt;kpi&gt;, Trees, Recovery board</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Priya, Admin</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Add a KPI
+2. Enter values and watch green, amber and red
+3. Build a formula and a tree
+4. Let a KPI drop to red
+5. Launch a recovery objective
+6. Move a threshold and see colours change</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M11</t>
+        </is>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A recovering KPI with its own objective</t>
+        </is>
+      </c>
+      <c r="I16" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nothing extra</t>
+        </is>
+      </c>
+      <c r="J16" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" ht="84" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M13 Initiatives, board and tasks</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Run the cycle</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Plan the work behind key results and move it on the board</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Initiatives, Initiatives / &lt;one&gt;, Board, Tasks / &lt;task&gt;</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mei, Sara, Priya, Admin</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Add an initiative and link it to a key result
+2. Add tasks on the board
+3. Drag cards between columns
+4. Watch a second browser update live
+5. Break a task into a checklist
+6. See the warning when done work moves nothing</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M11</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Work linked to key results, which the weekly session reads</t>
+        </is>
+      </c>
+      <c r="I17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two browsers side by side</t>
+        </is>
+      </c>
+      <c r="J17" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" ht="97" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M14 Check-in, review and inbox</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Run the cycle</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Report progress every week and have the reviewer acknowledge it</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check in, Review, Inbox</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sara, Priya, Mei, Jonas</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Sara opens what is due
+2. A check-in without a narrative is refused
+3. Sara posts one
+4. Others cannot post or acknowledge
+5. Priya acknowledges from Review
+6. Inbox: read, snooze, mute
+7. A stale goal turns Outdated</t>
+        </is>
+      </c>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M11</t>
+        </is>
+      </c>
+      <c r="H18" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check-ins and confidence the weekly session starts from</t>
+        </is>
+      </c>
+      <c r="I18" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check-in frequency set to daily so a goal is due today</t>
+        </is>
+      </c>
+      <c r="J18" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" ht="84" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M15 Weekly session</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Run the cycle</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run the four-step weekly session the product facilitates</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sessions, Session / &lt;id&gt;</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin (facilitator), Priya, Sara, Mei</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Start the template's weekly session
+2. Confidence round: vote, reveal, confirm
+3. A low key result needs a blocker
+4. Resolve and reassign the blocker
+5. Set two or three commitments
+6. Digest and close</t>
+        </is>
+      </c>
+      <c r="G19" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M14</t>
+        </is>
+      </c>
+      <c r="H19" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A finished session with blockers and commitments on record</t>
+        </is>
+      </c>
+      <c r="I19" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Priya and Sara are members of the session's space</t>
+        </is>
+      </c>
+      <c r="J19" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" ht="84" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M16 Agents and nudges</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Run the cycle</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check the two agents nudge, propose and stay quiet when they should</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin: Agents and runs, Nudge volume; Account, Where to reach you</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin, Sara</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Confirm both agents propose by default
+2. Run the Champion and the Coach now
+3. Apply and dismiss proposals
+4. Try sandbox and direct write
+5. A nudge reaches Sara once a day only
+6. Quiet hours and a switched-off rule hold nudges</t>
+        </is>
+      </c>
+      <c r="G20" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M14</t>
+        </is>
+      </c>
+      <c r="H20" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proof the agents are safe with AI off</t>
+        </is>
+      </c>
+      <c r="I20" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nothing extra</t>
+        </is>
+      </c>
+      <c r="J20" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" ht="84" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M17 Work map, search and activity</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5. Close and check</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check the overview screens, search and basic usability</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Work map, Search, Activity, copilot panel</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Priya, Jonas, Admin, Sara</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Read the work map strip and table
+2. Search finds only what you may open
+3. Page through Activity
+4. Open the copilot with AI off
+5. Check in with the keyboard only
+6. Use the app at phone width</t>
+        </is>
+      </c>
+      <c r="G21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M15</t>
+        </is>
+      </c>
+      <c r="H21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A read of the whole workspace as a member sees it</t>
+        </is>
+      </c>
+      <c r="I21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A phone, or a 375px browser window</t>
+        </is>
+      </c>
+      <c r="J21" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" ht="84" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M18 Closing the cycle and scorecard</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5. Close and check</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Close goals and the quarter, and record the result</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Goals / &lt;goal&gt;, Cycle phase 7, Scorecard, Cycles card</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sara, Admin</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Closing a goal needs a retrospective
+2. Close and reopen a goal
+3. Score every key result in phase 7
+4. Record the result on the scorecard
+5. Archive the old cycle
+6. Look for the quarterly review</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M15</t>
+        </is>
+      </c>
+      <c r="H22" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A closed cycle and a scorecard row</t>
+        </is>
+      </c>
+      <c r="I22" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nothing extra</t>
+        </is>
+      </c>
+      <c r="J22" s="1">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" ht="71" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M19 Access and permissions</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5. Close and check</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check nobody sees or does more than their access allows</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin screens, any goal URL, People / &lt;person&gt;</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jonas, Amara, Admin</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. A member opening Admin gets Not Found
+2. Signed-out visitors go to sign-in
+3. A hidden goal reads as not found
+4. Convert a member to a guest
+5. Erase a spare member</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M11</t>
+        </is>
+      </c>
+      <c r="H23" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Access control checked from the outside</t>
+        </is>
+      </c>
+      <c r="I23" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One spare invited account for erasing</t>
+        </is>
+      </c>
+      <c r="J23" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" ht="84" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M20 AI provider and copilot</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6. Integrations</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turn AI on and check it drafts while a person decides</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin, AI; drafting surface; copilot</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin, Sara, Jonas</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Store a provider key
+2. A bad key is marked invalid
+3. AI buttons appear
+4. A draft is proposed, not saved
+5. The copilot answers with sources
+6. Remove the key and the rules still fire</t>
+        </is>
+      </c>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M11</t>
+        </is>
+      </c>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AI checked on and off</t>
+        </is>
+      </c>
+      <c r="I24" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A provider key with a spending limit</t>
+        </is>
+      </c>
+      <c r="J24" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" ht="84" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M21 Chat channels and email</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6. Integrations</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deliver mail and chat messages to real inboxes and apps</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin, Channels; Account, Where to reach you</t>
+        </is>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin, Sara, Jonas</t>
+        </is>
+      </c>
+      <c r="F25" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Real mail arrives
+2. Connect Slack and link Sara
+3. A nudge arrives in Slack
+4. Chat commands work
+5. Repeat for Teams, WhatsApp, Telegram
+6. Disconnect a channel</t>
+        </is>
+      </c>
+      <c r="G25" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M16</t>
+        </is>
+      </c>
+      <c r="H25" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proof that reminders leave the product</t>
+        </is>
+      </c>
+      <c r="I25" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SMTP or Mailpit. A public URL and an app per chat provider</t>
+        </is>
+      </c>
+      <c r="J25" s="1">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26" ht="84" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M22 Single sign-on and directory sync</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6. Integrations</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sign in through a company identity provider and sync the directory</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin: Single sign-on, Directory sync, General</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin, Jonas</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Add an OIDC provider and restart
+2. Sign in with it
+3. Enforce SSO for a domain
+4. Try SAML
+5. Push a user through SCIM
+6. Require a second factor for everyone</t>
+        </is>
+      </c>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M04</t>
+        </is>
+      </c>
+      <c r="H26" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Company sign-in checked</t>
+        </is>
+      </c>
+      <c r="I26" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An identity provider account. Server access to restart</t>
+        </is>
+      </c>
+      <c r="J26" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="27" ht="84" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M23 Import and export</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6. Integrations</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bring data in from spreadsheets and FlowyTeam, and take it out</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin, Import</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Import goals from CSV
+2. Import the same file again: nothing new
+3. A bad row is reported
+4. Import KPI records from xlsx
+5. Export the workspace
+6. FlowyTeam import from the command line</t>
+        </is>
+      </c>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M07</t>
+        </is>
+      </c>
+      <c r="H27" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import and export checked</t>
+        </is>
+      </c>
+      <c r="I27" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sample CSV and xlsx files. A FlowyTeam MySQL copy for the last case</t>
+        </is>
+      </c>
+      <c r="J27" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="28" ht="71" customHeight="1">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M24 API tokens, CLI and external agents</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6. Integrations</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reach the product from scripts, the command line and outside AI agents</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account: API tokens, Device, Connected agents; /oauth/authorize</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sara</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Create and revoke a token
+2. Call the API with it
+3. Log the command line in by device approval
+4. Connect an MCP agent and ask it for goals
+5. Revoke the agent</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M11</t>
+        </is>
+      </c>
+      <c r="H28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The outside surfaces checked</t>
+        </is>
+      </c>
+      <c r="I28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The okr command line. An MCP client. A public HTTPS URL</t>
+        </is>
+      </c>
+      <c r="J28" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" ht="58" customHeight="1">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M25 Audit trail and workspace state</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6. Integrations</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check the audit trail recorded the sensitive actions from earlier modules</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin, Audit trail; Admin, General, State</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin, Sara</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Find the suspend and the publish override
+2. Verify the chain
+3. Export a date range
+4. Set the workspace read only, then active again</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M11</t>
+        </is>
+      </c>
+      <c r="H29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A verified audit trail</t>
+        </is>
+      </c>
+      <c r="I29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nothing extra</t>
+        </is>
+      </c>
+      <c r="J29" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" ht="71" customHeight="1">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M26 Cloud operator console</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6. Integrations</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check the managed-cloud operator console</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/operator, /operator/&lt;workspace&gt;, /operator/instance, Admin, Support access</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operator, Admin, Sara</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Console is hidden on self-hosted
+2. Operator lists workspaces
+3. Suspend and restore a workspace
+4. Ask for and approve support access
+5. Show an instance banner</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M04</t>
+        </is>
+      </c>
+      <c r="H30" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cloud operations checked</t>
+        </is>
+      </c>
+      <c r="I30" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OPENOKR_CLOUD=true and an operator row added by SQL</t>
+        </is>
+      </c>
+      <c r="J30" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total time</t>
+        </is>
+      </c>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="7"/>
+      <c r="J31" s="7">
+        <f>SUM(J5:J30)</f>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1591,7 +3223,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -1951,7 +3583,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -2045,7 +3677,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M01 Install and first account</t>
+          <t xml:space="preserve">M01 Install and first account: Turn an empty server into an instance with one owner. About 10 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B2" s="3"/>
@@ -2283,7 +3915,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M02 Welcome wizard</t>
+          <t xml:space="preserve">M02 Welcome wizard: Give the new workspace its name, clock, rhythm and starting content. Needs M01 first. About 10 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B7" s="3"/>
@@ -2474,7 +4106,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M03 Workspace settings</t>
+          <t xml:space="preserve">M03 Workspace settings: Check that workspace settings save, reload and reset. Needs M02 first. About 15 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B11" s="3"/>
@@ -2825,7 +4457,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M04 Invitations and building the team</t>
+          <t xml:space="preserve">M04 Invitations and building the team: Bring the seven Northwind people into the workspace. Needs M02 first. About 30 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B18" s="3"/>
@@ -3229,7 +4861,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M05 Sign-in and account security</t>
+          <t xml:space="preserve">M05 Sign-in and account security: Prove sign-in, password reset and the second factor protect an account. Needs M04 first. About 30 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B26" s="3"/>
@@ -3802,7 +5434,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M06 People and org chart</t>
+          <t xml:space="preserve">M06 People and org chart: Give everyone a title and a manager so the org chart is real. Needs M04 first. About 20 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B37" s="3"/>
@@ -4251,7 +5883,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M07 Spaces</t>
+          <t xml:space="preserve">M07 Spaces: Create the team homes that own goals, boards and sessions. Needs M06 first. About 20 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B46" s="3"/>
@@ -4593,7 +6225,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M08 Cycle: prepare, diagnose, direction</t>
+          <t xml:space="preserve">M08 Cycle: prepare, diagnose, direction: Walk the first three phases so drafting has something to stand on. Needs M07 first. About 25 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B53" s="3"/>
@@ -4939,7 +6571,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M09 Drafting OKRs and quality checks</t>
+          <t xml:space="preserve">M09 Drafting OKRs and quality checks: Draft objectives and key results while the quality checks fire live. Needs M08 first. About 40 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B60" s="3"/>
@@ -5700,7 +7332,7 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M10 Goal page and documents</t>
+          <t xml:space="preserve">M10 Goal page and documents: Work on one goal: values, confidence, comments, documents and files. Needs M09 first. About 30 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B75" s="3"/>
@@ -6261,7 +7893,7 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M11 Alignment and publishing</t>
+          <t xml:space="preserve">M11 Alignment and publishing: Align the set and publish it through the six gates. Needs M10 first. About 30 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B86" s="3"/>
@@ -6713,7 +8345,7 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M12 KPIs and recovery</t>
+          <t xml:space="preserve">M12 KPIs and recovery: Track KPIs continuously and recover one that falls out of its corridor. Needs M11 first. About 30 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B95" s="3"/>
@@ -7323,7 +8955,7 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M13 Initiatives, board and tasks</t>
+          <t xml:space="preserve">M13 Initiatives, board and tasks: Plan the work behind key results and move it on the board. Needs M11 first. About 30 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B107" s="3"/>
@@ -7826,7 +9458,7 @@
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M14 Check-in, review and inbox</t>
+          <t xml:space="preserve">M14 Check-in, review and inbox: Report progress every week and have the reviewer acknowledge it. Needs M11 first. About 30 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B117" s="3"/>
@@ -8435,7 +10067,7 @@
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M15 Weekly session</t>
+          <t xml:space="preserve">M15 Weekly session: Run the four-step weekly session the product facilitates. Needs M14 first. About 30 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B129" s="3"/>
@@ -8832,7 +10464,7 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M16 Agents and nudges</t>
+          <t xml:space="preserve">M16 Agents and nudges: Check the two agents nudge, propose and stay quiet when they should. Needs M14 first. About 30 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B137" s="3"/>
@@ -9439,7 +11071,7 @@
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M17 Work map, search and activity</t>
+          <t xml:space="preserve">M17 Work map, search and activity: Check the overview screens, search and basic usability. Needs M15 first. About 20 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B149" s="3"/>
@@ -9777,7 +11409,7 @@
     <row r="156">
       <c r="A156" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M18 Closing the cycle and scorecard</t>
+          <t xml:space="preserve">M18 Closing the cycle and scorecard: Close goals and the quarter, and record the result. Needs M15 first. About 25 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B156" s="3"/>
@@ -10120,7 +11752,7 @@
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M19 Access and permissions</t>
+          <t xml:space="preserve">M19 Access and permissions: Check nobody sees or does more than their access allows. Needs M11 first. About 15 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B163" s="3"/>
@@ -10412,7 +12044,7 @@
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M20 AI provider and copilot</t>
+          <t xml:space="preserve">M20 AI provider and copilot: Turn AI on and check it drafts while a person decides. Needs M11 first. About 30 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B169" s="3"/>
@@ -10858,7 +12490,7 @@
     <row r="178">
       <c r="A178" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M21 Chat channels and email</t>
+          <t xml:space="preserve">M21 Chat channels and email: Deliver mail and chat messages to real inboxes and apps. Needs M16 first. About 60 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B178" s="3"/>
@@ -11372,7 +13004,7 @@
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M22 Single sign-on and directory sync</t>
+          <t xml:space="preserve">M22 Single sign-on and directory sync: Sign in through a company identity provider and sync the directory. Needs M04 first. About 45 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B188" s="3"/>
@@ -11670,7 +13302,7 @@
     <row r="194">
       <c r="A194" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M23 Import and export</t>
+          <t xml:space="preserve">M23 Import and export: Bring data in from spreadsheets and FlowyTeam, and take it out. Needs M07 first. About 30 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B194" s="3"/>
@@ -12012,7 +13644,7 @@
     <row r="201">
       <c r="A201" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M24 API tokens, CLI and external agents</t>
+          <t xml:space="preserve">M24 API tokens, CLI and external agents: Reach the product from scripts, the command line and outside AI agents. Needs M11 first. About 30 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B201" s="3"/>
@@ -12250,7 +13882,7 @@
     <row r="206">
       <c r="A206" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M25 Audit trail and workspace state</t>
+          <t xml:space="preserve">M25 Audit trail and workspace state: Check the audit trail recorded the sensitive actions from earlier modules. Needs M11 first. About 15 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B206" s="3"/>
@@ -12481,7 +14113,7 @@
     <row r="211">
       <c r="A211" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">M26 Cloud operator console</t>
+          <t xml:space="preserve">M26 Cloud operator console: Check the managed-cloud operator console. Needs M04 first. About 30 min. Full workflow on the Module Guide sheet.</t>
         </is>
       </c>
       <c r="B211" s="3"/>
@@ -12799,7 +14431,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>

</xml_diff>

<commit_message>
H-21: the cloud can change a plan and grant its first operator
Nothing wrote a tenant's plan or seats after it was created, so no seat
limit could ever apply; the first operator needed hand-written SQL; and
S-49 had no seat list and no plan control.

- applyPlanInTx holds the one rule both sides keep: never below the
  headcount, refused naming both numbers. The plan's AI allowance becomes
  the workspace's monthly cost budget.
- workspace.changePlan for the administrator on S-49, which now shows the
  current plan and who holds each seat.
- setPlanAsOperator on S-46, with an optional seat count of the
  operator's own and a reason in the customer's audit log.
- pnpm cloud:operator grants and revokes the role: never self, only an
  operator grants the next, every change on the instance chain.

Signed-off-by: Akmal Akhpah <akmalakhpah@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/testing/OpenOKR-UAT.xlsx
+++ b/docs/testing/OpenOKR-UAT.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Bug Log" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test Cases'!$A$1:$N$218</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test Cases'!$A$1:$N$220</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Bug Log'!$A$1:$M$62</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -662,7 +662,7 @@
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generated from docs/testing/uat-cases.mjs and uat-guide.mjs. 191 test cases across 26 modules.</t>
+          <t xml:space="preserve">Generated from docs/testing/uat-cases.mjs and uat-guide.mjs. 193 test cases across 26 modules.</t>
         </is>
       </c>
       <c r="B86" s="10"/>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="I30" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPENOKR_CLOUD=true and an operator row added by SQL</t>
+          <t xml:space="preserve">OPENOKR_CLOUD=true and an operator granted with pnpm cloud:operator</t>
         </is>
       </c>
       <c r="J30" s="1">
@@ -14395,7 +14395,7 @@
       </c>
       <c r="E215" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPENOKR_CLOUD=true and the operator row added by SQL (docs/design/p8-t01b-operator-console.md)</t>
+          <t xml:space="preserve">OPENOKR_CLOUD=true and an operator granted with pnpm cloud:operator (docs/install/cloud.md)</t>
         </is>
       </c>
       <c r="F215" s="1" t="inlineStr">
@@ -14589,9 +14589,116 @@
       <c r="M218" s="5"/>
       <c r="N218" s="5"/>
     </row>
+    <row r="219">
+      <c r="A219" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M26-06</t>
+        </is>
+      </c>
+      <c r="B219" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M26 Cloud operator console</t>
+        </is>
+      </c>
+      <c r="C219" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operator sets a plan, and a downgrade below the headcount is refused</t>
+        </is>
+      </c>
+      <c r="D219" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operator</t>
+        </is>
+      </c>
+      <c r="E219" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M26-02 done, and cloud.plans holds a plan with fewer seats than Northwind Labs has people</t>
+        </is>
+      </c>
+      <c r="F219" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open the workspace, under "Plan and seats" pick the small plan, write a reason, click "Set the plan for Northwind Labs"
+2. Pick a larger plan, or type a seat count above the headcount, and apply again</t>
+        </is>
+      </c>
+      <c r="G219" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The first is refused naming the seats the plan has and the seats in use. The second is applied and the Tenant facts show the new plan and seats</t>
+        </is>
+      </c>
+      <c r="H219" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="I219" s="1"/>
+      <c r="J219" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="K219" s="5"/>
+      <c r="L219" s="5"/>
+      <c r="M219" s="5"/>
+      <c r="N219" s="5"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M26-07</t>
+        </is>
+      </c>
+      <c r="B220" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M26 Cloud operator console</t>
+        </is>
+      </c>
+      <c r="C220" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Administrator sees who holds a seat and changes plan</t>
+        </is>
+      </c>
+      <c r="D220" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin</t>
+        </is>
+      </c>
+      <c r="E220" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M26-07 done</t>
+        </is>
+      </c>
+      <c r="F220" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open Admin, Plan and seats
+2. Read the list under "Who holds a seat"
+3. Under "Move to" pick another plan and click "Change plan"</t>
+        </is>
+      </c>
+      <c r="G220" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The list names every person and invitation the seat count counts, and no guest or agent. The plan changes, or is refused naming both numbers when it has too few seats</t>
+        </is>
+      </c>
+      <c r="H220" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="I220" s="1"/>
+      <c r="J220" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Run</t>
+        </is>
+      </c>
+      <c r="K220" s="5"/>
+      <c r="L220" s="5"/>
+      <c r="M220" s="5"/>
+      <c r="N220" s="5"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N218"/>
-  <conditionalFormatting sqref="J2:J218">
+  <autoFilter ref="A1:N220"/>
+  <conditionalFormatting sqref="J2:J220">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",J2)))</formula>
     </cfRule>
@@ -14609,10 +14716,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J2:J218">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J2:J220">
       <formula1>"Not Run,Pass,Fail,Error,Blocked,N/A"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H2:H218">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H2:H220">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>